<commit_message>
day 1 solutions and streamlit
</commit_message>
<xml_diff>
--- a/docs/assets/RetirementPlan.xlsx
+++ b/docs/assets/RetirementPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerry\repos\mgmt675-2025\docs\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB8AC31-76DA-4B76-B3E0-0660A4CA2A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33179396-9E62-4869-B282-6F97091F3705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{5C29E880-E3A5-44DA-98FE-8F91E021F464}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{5C29E880-E3A5-44DA-98FE-8F91E021F464}"/>
   </bookViews>
   <sheets>
     <sheet name="Constant" sheetId="2" r:id="rId1"/>
@@ -79,9 +79,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -205,15 +206,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="4"/>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="4" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="3" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -224,46 +225,46 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -283,11 +284,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>14288</xdr:colOff>
+      <xdr:colOff>14287</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>4763</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6310312" cy="1600200"/>
+    <xdr:ext cx="6376987" cy="1600200"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
@@ -301,8 +302,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14288" y="3443288"/>
-          <a:ext cx="6310312" cy="1600200"/>
+          <a:off x="14287" y="3443288"/>
+          <a:ext cx="6376987" cy="1600200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -348,7 +349,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
-            <a:t> W for k years if</a:t>
+            <a:t> W for k years if account balance at end of year 5 equals PV of k years of withdrawals.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -357,7 +358,7 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
-            <a:t>PV(C + D for n years)  =  PV(W for k years) / (1+r)^n</a:t>
+            <a:t>FV at year n of C now + D for n years  =  PV at year n of W for k years</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -366,7 +367,7 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
-            <a:t>C + PV(D for n years)  =  W * PV(1 for k years) / (1+r)^n</a:t>
+            <a:t>C *(1+r)^n + FV(D for n years)  =  PV(W for k years)  =  W * PV(1 for k years) </a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -375,7 +376,23 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
-            <a:t>W  =  (1+r)^n * ( C + PV(D for n years) ) / (PV(1 for k years)</a:t>
+            <a:t>W  =  ( </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>C *(1+r)^n + FV(D for n years)  </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
+            <a:t>) / PV(1 for k years)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="1"/>
         </a:p>
@@ -391,18 +408,18 @@
   <autoFilter ref="A6:E16" xr:uid="{3F88EBF6-636E-45E1-A392-C661F36E012D}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{7409C94A-E697-44C7-9D7E-C22F02F76AF0}" name="Year"/>
-    <tableColumn id="2" xr3:uid="{ACC4C547-200E-4737-9F27-48D670883547}" name="Beginning Balance" totalsRowFunction="custom" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{ACC4C547-200E-4737-9F27-48D670883547}" name="Beginning Balance" totalsRowFunction="custom" dataDxfId="13">
       <totalsRowFormula>_xlfn.FORMULATEXT(B16)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{4EAF096E-91B3-4FED-B23F-1A6FBF35BFF6}" name="Return" totalsRowFunction="custom" dataDxfId="0" totalsRowDxfId="3">
+    <tableColumn id="3" xr3:uid="{4EAF096E-91B3-4FED-B23F-1A6FBF35BFF6}" name="Return" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
       <calculatedColumnFormula>$B$1</calculatedColumnFormula>
       <totalsRowFormula>_xlfn.FORMULATEXT(C16)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1C165765-58F8-404F-94FF-0449D6E68EF0}" name="Gain (Loss)" totalsRowFunction="custom" dataDxfId="5" totalsRowDxfId="2">
+    <tableColumn id="4" xr3:uid="{1C165765-58F8-404F-94FF-0449D6E68EF0}" name="Gain (Loss)" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
       <calculatedColumnFormula>Table13[[#This Row],[Beginning Balance]]*Table13[[#This Row],[Return]]</calculatedColumnFormula>
       <totalsRowFormula>_xlfn.FORMULATEXT(D7)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{62C0FD09-0B7C-48C9-B28E-12B5C3C01821}" name="Deposit (Withdrawal)" dataDxfId="4" totalsRowDxfId="1">
+    <tableColumn id="5" xr3:uid="{62C0FD09-0B7C-48C9-B28E-12B5C3C01821}" name="Deposit (Withdrawal)" dataDxfId="8" totalsRowDxfId="7">
       <calculatedColumnFormula>$B$3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -415,18 +432,18 @@
   <autoFilter ref="A8:E18" xr:uid="{3F88EBF6-636E-45E1-A392-C661F36E012D}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{9A8E175F-484A-45B5-9D47-DA340692B21E}" name="Year"/>
-    <tableColumn id="2" xr3:uid="{5650B33B-0DC4-44AC-95CB-32E7016ED274}" name="Beginning Balance" totalsRowFunction="custom" dataDxfId="10">
+    <tableColumn id="2" xr3:uid="{5650B33B-0DC4-44AC-95CB-32E7016ED274}" name="Beginning Balance" totalsRowFunction="custom" dataDxfId="6">
       <totalsRowFormula>_xlfn.FORMULATEXT(B18)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{79539066-3D2A-4F18-B9B6-23FF6E702527}" name="Return" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="9">
+    <tableColumn id="3" xr3:uid="{79539066-3D2A-4F18-B9B6-23FF6E702527}" name="Return" totalsRowFunction="custom" dataDxfId="5" totalsRowDxfId="4">
       <calculatedColumnFormula>IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</calculatedColumnFormula>
       <totalsRowFormula>_xlfn.FORMULATEXT(C18)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{08A68FFD-6E75-444F-B6D2-A3505D036DD3}" name="Gain (Loss)" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="8">
+    <tableColumn id="4" xr3:uid="{08A68FFD-6E75-444F-B6D2-A3505D036DD3}" name="Gain (Loss)" totalsRowFunction="custom" dataDxfId="3" totalsRowDxfId="2">
       <calculatedColumnFormula>Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</calculatedColumnFormula>
       <totalsRowFormula>_xlfn.FORMULATEXT(D9)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{32BA16FB-FDEB-462E-8343-1FE1469F03C9}" name="Deposit (Withdrawal)" dataDxfId="13" totalsRowDxfId="7">
+    <tableColumn id="5" xr3:uid="{32BA16FB-FDEB-462E-8343-1FE1469F03C9}" name="Deposit (Withdrawal)" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>$B$4</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -751,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E8EE5ED-AE51-483A-93BB-8617C3AD0B54}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.19921875" customWidth="1"/>
@@ -759,46 +776,48 @@
     <col min="3" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="17.3984375" customWidth="1"/>
     <col min="5" max="5" width="22.06640625" customWidth="1"/>
+    <col min="7" max="7" width="11.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="7">
+      <c r="B1" s="6">
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>50000</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>10000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10">
-        <f>(1+B1)^5*(PV(B1,5,-B3)+B2)/PV(B1,5,-1)</f>
+      <c r="B4" s="9">
+        <f>(B2*(1+B1)^5 + FV(B1,5,-B3))/PV(B1,5,-1)</f>
         <v>37347.524039737269</v>
       </c>
       <c r="C4" t="str">
         <f ca="1">_xlfn.FORMULATEXT(B4)</f>
-        <v>=(1+B1)^5*(PV(B1,5,-B3)+B2)/PV(B1,5,-1)</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+        <v>=(B2*(1+B1)^5 + FV(B1,5,-B3))/PV(B1,5,-1)</v>
+      </c>
+      <c r="G4" s="11"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -814,8 +833,9 @@
       <c r="E6" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="G6" s="11"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>1</v>
       </c>
@@ -836,7 +856,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2</v>
       </c>
@@ -856,8 +876,9 @@
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>3</v>
       </c>
@@ -878,7 +899,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>4</v>
       </c>
@@ -899,7 +920,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>5</v>
       </c>
@@ -920,7 +941,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>6</v>
       </c>
@@ -941,7 +962,7 @@
         <v>-37347.524039737269</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>7</v>
       </c>
@@ -962,7 +983,7 @@
         <v>-37347.524039737269</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>8</v>
       </c>
@@ -983,7 +1004,7 @@
         <v>-37347.524039737269</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1004,7 +1025,7 @@
         <v>-37347.524039737269</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1030,7 +1051,7 @@
         <f ca="1">_xlfn.FORMULATEXT(B16)</f>
         <v>=B15+D15+E15</v>
       </c>
-      <c r="C17" s="6" t="str">
+      <c r="C17" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C16)</f>
         <v>=$B$1</v>
       </c>
@@ -1071,50 +1092,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="7">
+      <c r="B1" s="6">
         <v>0.1</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>50000</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>10000</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>35000</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <v>0.1</v>
       </c>
     </row>
@@ -1145,11 +1166,11 @@
       </c>
       <c r="C9">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.21887911955466466</v>
+        <v>0.1937225788175708</v>
       </c>
       <c r="D9" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>10943.955977733232</v>
+        <v>9686.1289408785397</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" ref="E9:E13" si="0">$B$4</f>
@@ -1162,15 +1183,15 @@
       </c>
       <c r="B10" s="3">
         <f ca="1">B9+D9+E9</f>
-        <v>70943.955977733232</v>
+        <v>69686.128940878538</v>
       </c>
       <c r="C10">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>4.7393580971424543E-2</v>
+        <v>0.11818907640145628</v>
       </c>
       <c r="D10" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>3362.2881220638783</v>
+        <v>8236.1392175152268</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="0"/>
@@ -1183,15 +1204,15 @@
       </c>
       <c r="B11" s="3">
         <f t="shared" ref="B11:B18" ca="1" si="1">B10+D10+E10</f>
-        <v>84306.244099797113</v>
+        <v>87922.268158393766</v>
       </c>
       <c r="C11">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.27408022674978072</v>
+        <v>0.11658306975900531</v>
       </c>
       <c r="D11" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>23106.674499294757</v>
+        <v>10250.247922079992</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="0"/>
@@ -1204,15 +1225,15 @@
       </c>
       <c r="B12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>117412.91859909188</v>
+        <v>108172.51608047375</v>
       </c>
       <c r="C12">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.16827678812921243</v>
+        <v>9.2251242334983552E-2</v>
       </c>
       <c r="D12" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>19757.86882673185</v>
+        <v>9979.0489949246894</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="0"/>
@@ -1225,15 +1246,15 @@
       </c>
       <c r="B13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>147170.78742582374</v>
+        <v>128151.56507539844</v>
       </c>
       <c r="C13">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.16071808284883557</v>
+        <v>0.51979829770178376</v>
       </c>
       <c r="D13" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>23653.006806431909</v>
+        <v>66612.965374011474</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" si="0"/>
@@ -1246,15 +1267,15 @@
       </c>
       <c r="B14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>180823.79423225566</v>
+        <v>204764.53044940991</v>
       </c>
       <c r="C14">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.171654817955714</v>
+        <v>0.11112905439480462</v>
       </c>
       <c r="D14" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>31039.275480999331</v>
+        <v>22755.288642439104</v>
       </c>
       <c r="E14" s="3">
         <f>-$B$5</f>
@@ -1267,15 +1288,15 @@
       </c>
       <c r="B15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>176863.06971325498</v>
+        <v>192519.81909184903</v>
       </c>
       <c r="C15">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.15284381720892876</v>
+        <v>-0.17841391976643053</v>
       </c>
       <c r="D15" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>27032.426698262767</v>
+        <v>-34348.215556900876</v>
       </c>
       <c r="E15" s="3">
         <f>-$B$5</f>
@@ -1288,15 +1309,15 @@
       </c>
       <c r="B16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>168895.49641151776</v>
+        <v>123171.60353494814</v>
       </c>
       <c r="C16">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>0.27193135914600908</v>
+        <v>0.50748058904602511</v>
       </c>
       <c r="D16" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>45927.981892823926</v>
+        <v>62507.197915658951</v>
       </c>
       <c r="E16" s="3">
         <f t="shared" ref="E16:E18" si="2">-$B$5</f>
@@ -1309,15 +1330,15 @@
       </c>
       <c r="B17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>179823.47830434167</v>
+        <v>150678.80145060708</v>
       </c>
       <c r="C17">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>-5.7464762305794725E-2</v>
+        <v>5.9650166804658733E-2</v>
       </c>
       <c r="D17" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>-10333.513437760228</v>
+        <v>8988.015640454767</v>
       </c>
       <c r="E17" s="3">
         <f t="shared" si="2"/>
@@ -1330,15 +1351,15 @@
       </c>
       <c r="B18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>134489.96486658143</v>
+        <v>124666.81709106185</v>
       </c>
       <c r="C18">
         <f ca="1">IF(Table1[[#This Row],[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</f>
-        <v>-2.6415683050026784E-2</v>
+        <v>-0.13080234406365143</v>
       </c>
       <c r="D18" s="3">
         <f ca="1">Table1[[#This Row],[Beginning Balance]]*Table1[[#This Row],[Return]]</f>
-        <v>-3552.6442853248527</v>
+        <v>-16306.711902465373</v>
       </c>
       <c r="E18" s="3">
         <f t="shared" si="2"/>
@@ -1350,7 +1371,7 @@
         <f ca="1">_xlfn.FORMULATEXT(B18)</f>
         <v>=B17+D17+E17</v>
       </c>
-      <c r="C19" s="6" t="str">
+      <c r="C19" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C18)</f>
         <v>=IF([@[Beginning Balance]]&gt;0, NORMINV(RAND(), $B$1, $B$2), $B$6)</v>
       </c>
@@ -1366,7 +1387,7 @@
       </c>
       <c r="B20" s="5">
         <f ca="1">B18+D18+E18</f>
-        <v>95937.320581256572</v>
+        <v>73360.10518859647</v>
       </c>
     </row>
   </sheetData>

</xml_diff>